<commit_message>
chore: cap nhat Masterlist 2027-2028_Mau.xlsx
</commit_message>
<xml_diff>
--- a/Masterlist 2027-2028_Mau.xlsx
+++ b/Masterlist 2027-2028_Mau.xlsx
@@ -5,20 +5,21 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\QHDC3\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\QHDC3\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="7440" yWindow="0" windowWidth="19200" windowHeight="7050" tabRatio="659" activeTab="3"/>
+    <workbookView xWindow="8490" yWindow="0" windowWidth="19200" windowHeight="7050" tabRatio="659" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="PL1.1 ML2027-2028" sheetId="1" r:id="rId1"/>
     <sheet name="TH theo DV" sheetId="14" r:id="rId2"/>
     <sheet name="TH theo Mảng" sheetId="20" r:id="rId3"/>
     <sheet name="TH theo Dịch vụ" sheetId="21" r:id="rId4"/>
-    <sheet name="PL1.2 TH theo mục đích" sheetId="18" state="hidden" r:id="rId5"/>
-    <sheet name="PL1.3 Buc tranh sau QH" sheetId="4" state="hidden" r:id="rId6"/>
-    <sheet name="Mã" sheetId="15" state="hidden" r:id="rId7"/>
+    <sheet name="So sanh CL" sheetId="22" r:id="rId5"/>
+    <sheet name="PL1.2 TH theo mục đích" sheetId="18" state="hidden" r:id="rId6"/>
+    <sheet name="PL1.3 Buc tranh sau QH" sheetId="4" state="hidden" r:id="rId7"/>
+    <sheet name="Mã" sheetId="15" state="hidden" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="\p">#REF!</definedName>
@@ -107,8 +108,8 @@
     <definedName name="_Fill" localSheetId="0" hidden="1">#REF!</definedName>
     <definedName name="_Fill" hidden="1">#REF!</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'PL1.1 ML2027-2028'!$A$7:$Q$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'PL1.2 TH theo mục đích'!$A$5:$K$57</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PL1.3 Buc tranh sau QH'!$A$3:$G$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PL1.2 TH theo mục đích'!$A$5:$K$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'PL1.3 Buc tranh sau QH'!$A$3:$G$29</definedName>
     <definedName name="_xlnm._FilterDatabase" hidden="1">#REF!</definedName>
     <definedName name="_H500866">#REF!</definedName>
     <definedName name="_kbps_sub_ATT_DCOM_3G">#REF!</definedName>
@@ -698,13 +699,13 @@
     <definedName name="PRICE">#REF!</definedName>
     <definedName name="PRICE1">#REF!</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'PL1.1 ML2027-2028'!$A$1:$I$10</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'PL1.2 TH theo mục đích'!$A$1:$J$58</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'PL1.3 Buc tranh sau QH'!$A$1:$F$29</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="5">'PL1.2 TH theo mục đích'!$A$1:$J$58</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'PL1.3 Buc tranh sau QH'!$A$1:$F$29</definedName>
     <definedName name="_xlnm.Print_Area">#REF!</definedName>
     <definedName name="PRINT_AREA_MI">#REF!</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'PL1.1 ML2027-2028'!$4:$7</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="4">'PL1.2 TH theo mục đích'!$3:$4</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="5">'PL1.3 Buc tranh sau QH'!$3:$3</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'PL1.2 TH theo mục đích'!$3:$4</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'PL1.3 Buc tranh sau QH'!$3:$3</definedName>
     <definedName name="_xlnm.Print_Titles">#N/A</definedName>
     <definedName name="PRINT_TITLES_MI">#REF!</definedName>
     <definedName name="PRINTA">#REF!</definedName>
@@ -966,7 +967,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="981" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="363">
   <si>
     <t>TT</t>
   </si>
@@ -2212,6 +2213,39 @@
   </si>
   <si>
     <t>PM</t>
+  </si>
+  <si>
+    <t>MẢNG / LĨNH VỰC</t>
+  </si>
+  <si>
+    <t>CHIẾN LƯỢC 5 NĂM (M$)</t>
+  </si>
+  <si>
+    <t>TỔNG</t>
+  </si>
+  <si>
+    <t>QHĐC 2027-2028 (M$)</t>
+  </si>
+  <si>
+    <t>CHÊNH LỆCH SO VỚI CHIẾN LƯỢC (M$)</t>
+  </si>
+  <si>
+    <t>Công nghệ thông tin</t>
+  </si>
+  <si>
+    <t>Cơ điện tổng trạm</t>
+  </si>
+  <si>
+    <t>Cơ điện BTS</t>
+  </si>
+  <si>
+    <t>Tổng (m$)</t>
+  </si>
+  <si>
+    <t>Phần mềm, công cụ</t>
+  </si>
+  <si>
+    <t>BRCĐ-TH</t>
   </si>
 </sst>
 </file>
@@ -2627,7 +2661,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2733,6 +2767,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0" tint="-4.9989318521683403E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3312,7 +3352,7 @@
     <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="662">
+  <cellXfs count="672">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5149,41 +5189,95 @@
     <xf numFmtId="0" fontId="24" fillId="10" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="40" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="50" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="50" fillId="18" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="18" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="18" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="50" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -5191,60 +5285,6 @@
     <xf numFmtId="0" fontId="50" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="56" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="55" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="18" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="18" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="50" fillId="18" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="18" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5278,6 +5318,30 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="19" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="37" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="37" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="290">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -10051,15 +10115,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:19" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B1" s="619" t="s">
+      <c r="B1" s="629" t="s">
         <v>214</v>
       </c>
-      <c r="C1" s="619"/>
-      <c r="D1" s="619"/>
-      <c r="E1" s="619"/>
-      <c r="F1" s="619"/>
-      <c r="G1" s="619"/>
-      <c r="H1" s="619"/>
+      <c r="C1" s="629"/>
+      <c r="D1" s="629"/>
+      <c r="E1" s="629"/>
+      <c r="F1" s="629"/>
+      <c r="G1" s="629"/>
+      <c r="H1" s="629"/>
     </row>
     <row r="2" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B2" s="357" t="s">
@@ -10067,51 +10131,51 @@
       </c>
     </row>
     <row r="3" spans="2:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="620" t="s">
+      <c r="B3" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="621" t="s">
+      <c r="C3" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D3" s="621" t="s">
+      <c r="D3" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="621">
+      <c r="E3" s="619">
         <v>2027</v>
       </c>
-      <c r="F3" s="621">
+      <c r="F3" s="619">
         <v>2028</v>
       </c>
-      <c r="G3" s="621" t="s">
+      <c r="G3" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H3" s="621"/>
+      <c r="H3" s="619"/>
       <c r="I3" s="502"/>
-      <c r="J3" s="620" t="s">
+      <c r="J3" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="K3" s="621" t="s">
+      <c r="K3" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="L3" s="621" t="s">
+      <c r="L3" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="M3" s="621"/>
-      <c r="N3" s="621"/>
-      <c r="O3" s="621"/>
-      <c r="P3" s="621"/>
-      <c r="Q3" s="621"/>
-      <c r="R3" s="629" t="s">
+      <c r="M3" s="619"/>
+      <c r="N3" s="619"/>
+      <c r="O3" s="619"/>
+      <c r="P3" s="619"/>
+      <c r="Q3" s="619"/>
+      <c r="R3" s="620" t="s">
         <v>218</v>
       </c>
       <c r="S3" s="356"/>
     </row>
     <row r="4" spans="2:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="620"/>
-      <c r="C4" s="621"/>
-      <c r="D4" s="621"/>
-      <c r="E4" s="621"/>
-      <c r="F4" s="621"/>
+      <c r="B4" s="628"/>
+      <c r="C4" s="619"/>
+      <c r="D4" s="619"/>
+      <c r="E4" s="619"/>
+      <c r="F4" s="619"/>
       <c r="G4" s="583">
         <v>2027</v>
       </c>
@@ -10119,8 +10183,8 @@
         <v>2028</v>
       </c>
       <c r="I4" s="502"/>
-      <c r="J4" s="620"/>
-      <c r="K4" s="621"/>
+      <c r="J4" s="628"/>
+      <c r="K4" s="619"/>
       <c r="L4" s="503" t="s">
         <v>41</v>
       </c>
@@ -10139,7 +10203,7 @@
       <c r="Q4" s="358">
         <v>2030</v>
       </c>
-      <c r="R4" s="630"/>
+      <c r="R4" s="621"/>
       <c r="S4" s="356"/>
     </row>
     <row r="5" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
@@ -10551,45 +10615,45 @@
       <c r="Q14" s="367"/>
     </row>
     <row r="15" spans="2:19" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="620" t="s">
+      <c r="B15" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="621" t="s">
+      <c r="C15" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D15" s="621" t="s">
+      <c r="D15" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="621">
+      <c r="E15" s="619">
         <v>2027</v>
       </c>
-      <c r="F15" s="621">
+      <c r="F15" s="619">
         <v>2028</v>
       </c>
-      <c r="G15" s="621" t="s">
+      <c r="G15" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H15" s="621"/>
+      <c r="H15" s="619"/>
       <c r="I15" s="502"/>
-      <c r="J15" s="621" t="s">
+      <c r="J15" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K15" s="621"/>
-      <c r="L15" s="621"/>
-      <c r="M15" s="621"/>
-      <c r="N15" s="621"/>
-      <c r="O15" s="621"/>
-      <c r="P15" s="629" t="s">
+      <c r="K15" s="619"/>
+      <c r="L15" s="619"/>
+      <c r="M15" s="619"/>
+      <c r="N15" s="619"/>
+      <c r="O15" s="619"/>
+      <c r="P15" s="620" t="s">
         <v>218</v>
       </c>
       <c r="Q15" s="367"/>
     </row>
     <row r="16" spans="2:19" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="620"/>
-      <c r="C16" s="621"/>
-      <c r="D16" s="621"/>
-      <c r="E16" s="621"/>
-      <c r="F16" s="621"/>
+      <c r="B16" s="628"/>
+      <c r="C16" s="619"/>
+      <c r="D16" s="619"/>
+      <c r="E16" s="619"/>
+      <c r="F16" s="619"/>
       <c r="G16" s="583">
         <v>2027</v>
       </c>
@@ -10615,7 +10679,7 @@
       <c r="O16" s="374">
         <v>2030</v>
       </c>
-      <c r="P16" s="630"/>
+      <c r="P16" s="621"/>
       <c r="Q16" s="367"/>
     </row>
     <row r="17" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
@@ -10904,45 +10968,45 @@
       <c r="Q24" s="367"/>
     </row>
     <row r="25" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="620" t="s">
+      <c r="B25" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="621" t="s">
+      <c r="C25" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D25" s="621" t="s">
+      <c r="D25" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E25" s="621">
+      <c r="E25" s="619">
         <v>2027</v>
       </c>
-      <c r="F25" s="621">
+      <c r="F25" s="619">
         <v>2028</v>
       </c>
-      <c r="G25" s="621" t="s">
+      <c r="G25" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H25" s="621"/>
+      <c r="H25" s="619"/>
       <c r="I25" s="502"/>
-      <c r="J25" s="621" t="s">
+      <c r="J25" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K25" s="621"/>
-      <c r="L25" s="621"/>
-      <c r="M25" s="621"/>
-      <c r="N25" s="621"/>
-      <c r="O25" s="621"/>
-      <c r="P25" s="629" t="s">
+      <c r="K25" s="619"/>
+      <c r="L25" s="619"/>
+      <c r="M25" s="619"/>
+      <c r="N25" s="619"/>
+      <c r="O25" s="619"/>
+      <c r="P25" s="620" t="s">
         <v>218</v>
       </c>
       <c r="Q25" s="367"/>
     </row>
     <row r="26" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B26" s="620"/>
-      <c r="C26" s="621"/>
-      <c r="D26" s="621"/>
-      <c r="E26" s="621"/>
-      <c r="F26" s="621"/>
+      <c r="B26" s="628"/>
+      <c r="C26" s="619"/>
+      <c r="D26" s="619"/>
+      <c r="E26" s="619"/>
+      <c r="F26" s="619"/>
       <c r="G26" s="583">
         <v>2027</v>
       </c>
@@ -10968,7 +11032,7 @@
       <c r="O26" s="374">
         <v>2030</v>
       </c>
-      <c r="P26" s="630"/>
+      <c r="P26" s="621"/>
       <c r="Q26" s="367"/>
     </row>
     <row r="27" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
@@ -11245,45 +11309,45 @@
       <c r="Q34" s="367"/>
     </row>
     <row r="35" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B35" s="620" t="s">
+      <c r="B35" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C35" s="621" t="s">
+      <c r="C35" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D35" s="621" t="s">
+      <c r="D35" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E35" s="621">
+      <c r="E35" s="619">
         <v>2027</v>
       </c>
-      <c r="F35" s="621">
+      <c r="F35" s="619">
         <v>2028</v>
       </c>
-      <c r="G35" s="621" t="s">
+      <c r="G35" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H35" s="621"/>
+      <c r="H35" s="619"/>
       <c r="I35" s="502"/>
-      <c r="J35" s="621" t="s">
+      <c r="J35" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K35" s="621"/>
-      <c r="L35" s="621"/>
-      <c r="M35" s="621"/>
-      <c r="N35" s="621"/>
-      <c r="O35" s="621"/>
-      <c r="P35" s="629" t="s">
+      <c r="K35" s="619"/>
+      <c r="L35" s="619"/>
+      <c r="M35" s="619"/>
+      <c r="N35" s="619"/>
+      <c r="O35" s="619"/>
+      <c r="P35" s="620" t="s">
         <v>246</v>
       </c>
       <c r="Q35" s="367"/>
     </row>
     <row r="36" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B36" s="620"/>
-      <c r="C36" s="621"/>
-      <c r="D36" s="621"/>
-      <c r="E36" s="621"/>
-      <c r="F36" s="621"/>
+      <c r="B36" s="628"/>
+      <c r="C36" s="619"/>
+      <c r="D36" s="619"/>
+      <c r="E36" s="619"/>
+      <c r="F36" s="619"/>
       <c r="G36" s="583">
         <v>2027</v>
       </c>
@@ -11309,7 +11373,7 @@
       <c r="O36" s="374">
         <v>2030</v>
       </c>
-      <c r="P36" s="630"/>
+      <c r="P36" s="621"/>
       <c r="Q36" s="367"/>
     </row>
     <row r="37" spans="2:17" x14ac:dyDescent="0.25">
@@ -11633,45 +11697,45 @@
       <c r="Q45" s="367"/>
     </row>
     <row r="46" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B46" s="620" t="s">
+      <c r="B46" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C46" s="621" t="s">
+      <c r="C46" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D46" s="621" t="s">
+      <c r="D46" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E46" s="621">
+      <c r="E46" s="619">
         <v>2027</v>
       </c>
-      <c r="F46" s="621">
+      <c r="F46" s="619">
         <v>2028</v>
       </c>
-      <c r="G46" s="621" t="s">
+      <c r="G46" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H46" s="621"/>
+      <c r="H46" s="619"/>
       <c r="I46" s="502"/>
-      <c r="J46" s="621" t="s">
+      <c r="J46" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K46" s="621"/>
-      <c r="L46" s="621"/>
-      <c r="M46" s="621"/>
-      <c r="N46" s="621"/>
-      <c r="O46" s="621"/>
-      <c r="P46" s="628" t="s">
+      <c r="K46" s="619"/>
+      <c r="L46" s="619"/>
+      <c r="M46" s="619"/>
+      <c r="N46" s="619"/>
+      <c r="O46" s="619"/>
+      <c r="P46" s="623" t="s">
         <v>246</v>
       </c>
       <c r="Q46" s="367"/>
     </row>
     <row r="47" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B47" s="620"/>
-      <c r="C47" s="621"/>
-      <c r="D47" s="621"/>
-      <c r="E47" s="621"/>
-      <c r="F47" s="621"/>
+      <c r="B47" s="628"/>
+      <c r="C47" s="619"/>
+      <c r="D47" s="619"/>
+      <c r="E47" s="619"/>
+      <c r="F47" s="619"/>
       <c r="G47" s="583">
         <v>2027</v>
       </c>
@@ -11697,7 +11761,7 @@
       <c r="O47" s="358">
         <v>2030</v>
       </c>
-      <c r="P47" s="628"/>
+      <c r="P47" s="623"/>
       <c r="Q47" s="367"/>
     </row>
     <row r="48" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
@@ -12140,55 +12204,55 @@
       <c r="Q58" s="367"/>
     </row>
     <row r="59" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B59" s="622" t="s">
+      <c r="B59" s="630" t="s">
         <v>271</v>
       </c>
-      <c r="C59" s="622"/>
-      <c r="D59" s="622"/>
-      <c r="E59" s="622"/>
-      <c r="F59" s="622"/>
+      <c r="C59" s="630"/>
+      <c r="D59" s="630"/>
+      <c r="E59" s="630"/>
+      <c r="F59" s="630"/>
       <c r="Q59" s="367"/>
     </row>
     <row r="60" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B60" s="620" t="s">
+      <c r="B60" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C60" s="621" t="s">
+      <c r="C60" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D60" s="621" t="s">
+      <c r="D60" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E60" s="621">
+      <c r="E60" s="619">
         <v>2027</v>
       </c>
-      <c r="F60" s="621">
+      <c r="F60" s="619">
         <v>2028</v>
       </c>
-      <c r="G60" s="621" t="s">
+      <c r="G60" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H60" s="621"/>
+      <c r="H60" s="619"/>
       <c r="I60" s="502"/>
-      <c r="J60" s="621" t="s">
+      <c r="J60" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K60" s="621"/>
-      <c r="L60" s="621"/>
-      <c r="M60" s="621"/>
-      <c r="N60" s="621"/>
-      <c r="O60" s="621"/>
-      <c r="P60" s="629" t="s">
+      <c r="K60" s="619"/>
+      <c r="L60" s="619"/>
+      <c r="M60" s="619"/>
+      <c r="N60" s="619"/>
+      <c r="O60" s="619"/>
+      <c r="P60" s="620" t="s">
         <v>218</v>
       </c>
       <c r="Q60" s="367"/>
     </row>
     <row r="61" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B61" s="620"/>
-      <c r="C61" s="621"/>
-      <c r="D61" s="621"/>
-      <c r="E61" s="621"/>
-      <c r="F61" s="621"/>
+      <c r="B61" s="628"/>
+      <c r="C61" s="619"/>
+      <c r="D61" s="619"/>
+      <c r="E61" s="619"/>
+      <c r="F61" s="619"/>
       <c r="G61" s="583">
         <v>2027</v>
       </c>
@@ -12214,7 +12278,7 @@
       <c r="O61" s="358">
         <v>2030</v>
       </c>
-      <c r="P61" s="630"/>
+      <c r="P61" s="621"/>
       <c r="Q61" s="367"/>
     </row>
     <row r="62" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
@@ -12616,45 +12680,45 @@
       <c r="Q72" s="367"/>
     </row>
     <row r="73" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B73" s="620" t="s">
+      <c r="B73" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C73" s="621" t="s">
+      <c r="C73" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D73" s="621" t="s">
+      <c r="D73" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E73" s="621">
+      <c r="E73" s="619">
         <v>2027</v>
       </c>
-      <c r="F73" s="621">
+      <c r="F73" s="619">
         <v>2028</v>
       </c>
-      <c r="G73" s="621" t="s">
+      <c r="G73" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H73" s="621"/>
+      <c r="H73" s="619"/>
       <c r="I73" s="502"/>
-      <c r="J73" s="621" t="s">
+      <c r="J73" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K73" s="621"/>
-      <c r="L73" s="621"/>
-      <c r="M73" s="621"/>
-      <c r="N73" s="621"/>
-      <c r="O73" s="621"/>
-      <c r="P73" s="627" t="s">
+      <c r="K73" s="619"/>
+      <c r="L73" s="619"/>
+      <c r="M73" s="619"/>
+      <c r="N73" s="619"/>
+      <c r="O73" s="619"/>
+      <c r="P73" s="622" t="s">
         <v>218</v>
       </c>
       <c r="Q73" s="367"/>
     </row>
     <row r="74" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B74" s="620"/>
-      <c r="C74" s="621"/>
-      <c r="D74" s="621"/>
-      <c r="E74" s="621"/>
-      <c r="F74" s="621"/>
+      <c r="B74" s="628"/>
+      <c r="C74" s="619"/>
+      <c r="D74" s="619"/>
+      <c r="E74" s="619"/>
+      <c r="F74" s="619"/>
       <c r="G74" s="583">
         <v>2027</v>
       </c>
@@ -12680,7 +12744,7 @@
       <c r="O74" s="412">
         <v>2030</v>
       </c>
-      <c r="P74" s="627"/>
+      <c r="P74" s="622"/>
       <c r="Q74" s="367"/>
     </row>
     <row r="75" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
@@ -12857,52 +12921,52 @@
       <c r="Q79" s="367"/>
     </row>
     <row r="80" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B80" s="623" t="s">
+      <c r="B80" s="624" t="s">
         <v>290</v>
       </c>
-      <c r="C80" s="623"/>
+      <c r="C80" s="624"/>
       <c r="Q80" s="367"/>
     </row>
     <row r="81" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B81" s="620" t="s">
+      <c r="B81" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C81" s="621" t="s">
+      <c r="C81" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D81" s="621" t="s">
+      <c r="D81" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E81" s="621">
+      <c r="E81" s="619">
         <v>2027</v>
       </c>
-      <c r="F81" s="621">
+      <c r="F81" s="619">
         <v>2028</v>
       </c>
-      <c r="G81" s="621" t="s">
+      <c r="G81" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H81" s="621"/>
+      <c r="H81" s="619"/>
       <c r="I81" s="502"/>
-      <c r="J81" s="621" t="s">
+      <c r="J81" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K81" s="621"/>
-      <c r="L81" s="621"/>
-      <c r="M81" s="621"/>
-      <c r="N81" s="621"/>
-      <c r="O81" s="621"/>
-      <c r="P81" s="627" t="s">
+      <c r="K81" s="619"/>
+      <c r="L81" s="619"/>
+      <c r="M81" s="619"/>
+      <c r="N81" s="619"/>
+      <c r="O81" s="619"/>
+      <c r="P81" s="622" t="s">
         <v>218</v>
       </c>
       <c r="Q81" s="367"/>
     </row>
     <row r="82" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B82" s="620"/>
-      <c r="C82" s="621"/>
-      <c r="D82" s="621"/>
-      <c r="E82" s="621"/>
-      <c r="F82" s="621"/>
+      <c r="B82" s="628"/>
+      <c r="C82" s="619"/>
+      <c r="D82" s="619"/>
+      <c r="E82" s="619"/>
+      <c r="F82" s="619"/>
       <c r="G82" s="583">
         <v>2027</v>
       </c>
@@ -12928,7 +12992,7 @@
       <c r="O82" s="412">
         <v>2030</v>
       </c>
-      <c r="P82" s="627"/>
+      <c r="P82" s="622"/>
       <c r="Q82" s="367"/>
     </row>
     <row r="83" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
@@ -13353,45 +13417,45 @@
       <c r="Q93" s="367"/>
     </row>
     <row r="94" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B94" s="620" t="s">
+      <c r="B94" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C94" s="621" t="s">
+      <c r="C94" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D94" s="621" t="s">
+      <c r="D94" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E94" s="621">
+      <c r="E94" s="619">
         <v>2027</v>
       </c>
-      <c r="F94" s="621">
+      <c r="F94" s="619">
         <v>2028</v>
       </c>
-      <c r="G94" s="621" t="s">
+      <c r="G94" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H94" s="621"/>
+      <c r="H94" s="619"/>
       <c r="I94" s="502"/>
-      <c r="J94" s="621" t="s">
+      <c r="J94" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K94" s="621"/>
-      <c r="L94" s="621"/>
-      <c r="M94" s="621"/>
-      <c r="N94" s="621"/>
-      <c r="O94" s="621"/>
-      <c r="P94" s="624" t="s">
+      <c r="K94" s="619"/>
+      <c r="L94" s="619"/>
+      <c r="M94" s="619"/>
+      <c r="N94" s="619"/>
+      <c r="O94" s="619"/>
+      <c r="P94" s="625" t="s">
         <v>218</v>
       </c>
       <c r="Q94" s="367"/>
     </row>
     <row r="95" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B95" s="620"/>
-      <c r="C95" s="621"/>
-      <c r="D95" s="621"/>
-      <c r="E95" s="621"/>
-      <c r="F95" s="621"/>
+      <c r="B95" s="628"/>
+      <c r="C95" s="619"/>
+      <c r="D95" s="619"/>
+      <c r="E95" s="619"/>
+      <c r="F95" s="619"/>
       <c r="G95" s="583">
         <v>2027</v>
       </c>
@@ -13417,7 +13481,7 @@
       <c r="O95" s="431">
         <v>2030</v>
       </c>
-      <c r="P95" s="626"/>
+      <c r="P95" s="627"/>
       <c r="Q95" s="367"/>
     </row>
     <row r="96" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
@@ -13832,53 +13896,53 @@
       <c r="Q105" s="367"/>
     </row>
     <row r="106" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B106" s="623" t="s">
+      <c r="B106" s="624" t="s">
         <v>302</v>
       </c>
-      <c r="C106" s="623"/>
-      <c r="D106" s="623"/>
+      <c r="C106" s="624"/>
+      <c r="D106" s="624"/>
       <c r="Q106" s="367"/>
     </row>
     <row r="107" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B107" s="620" t="s">
+      <c r="B107" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C107" s="621" t="s">
+      <c r="C107" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D107" s="621" t="s">
+      <c r="D107" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E107" s="621">
+      <c r="E107" s="619">
         <v>2027</v>
       </c>
-      <c r="F107" s="621">
+      <c r="F107" s="619">
         <v>2028</v>
       </c>
-      <c r="G107" s="621" t="s">
+      <c r="G107" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H107" s="621"/>
+      <c r="H107" s="619"/>
       <c r="I107" s="502"/>
-      <c r="J107" s="621" t="s">
+      <c r="J107" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K107" s="621"/>
-      <c r="L107" s="621"/>
-      <c r="M107" s="621"/>
-      <c r="N107" s="621"/>
-      <c r="O107" s="621"/>
-      <c r="P107" s="624" t="s">
+      <c r="K107" s="619"/>
+      <c r="L107" s="619"/>
+      <c r="M107" s="619"/>
+      <c r="N107" s="619"/>
+      <c r="O107" s="619"/>
+      <c r="P107" s="625" t="s">
         <v>218</v>
       </c>
       <c r="Q107" s="367"/>
     </row>
     <row r="108" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B108" s="620"/>
-      <c r="C108" s="621"/>
-      <c r="D108" s="621"/>
-      <c r="E108" s="621"/>
-      <c r="F108" s="621"/>
+      <c r="B108" s="628"/>
+      <c r="C108" s="619"/>
+      <c r="D108" s="619"/>
+      <c r="E108" s="619"/>
+      <c r="F108" s="619"/>
       <c r="G108" s="583">
         <v>2027</v>
       </c>
@@ -13904,7 +13968,7 @@
       <c r="O108" s="431">
         <v>2030</v>
       </c>
-      <c r="P108" s="626"/>
+      <c r="P108" s="627"/>
       <c r="Q108" s="367"/>
     </row>
     <row r="109" spans="2:17" ht="30" x14ac:dyDescent="0.25">
@@ -13950,53 +14014,53 @@
       <c r="Q110" s="367"/>
     </row>
     <row r="111" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B111" s="623" t="s">
+      <c r="B111" s="624" t="s">
         <v>305</v>
       </c>
-      <c r="C111" s="623"/>
-      <c r="D111" s="623"/>
+      <c r="C111" s="624"/>
+      <c r="D111" s="624"/>
       <c r="Q111" s="367"/>
     </row>
     <row r="112" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B112" s="620" t="s">
+      <c r="B112" s="628" t="s">
         <v>48</v>
       </c>
-      <c r="C112" s="621" t="s">
+      <c r="C112" s="619" t="s">
         <v>216</v>
       </c>
-      <c r="D112" s="621" t="s">
+      <c r="D112" s="619" t="s">
         <v>41</v>
       </c>
-      <c r="E112" s="621">
+      <c r="E112" s="619">
         <v>2027</v>
       </c>
-      <c r="F112" s="621">
+      <c r="F112" s="619">
         <v>2028</v>
       </c>
-      <c r="G112" s="621" t="s">
+      <c r="G112" s="619" t="s">
         <v>218</v>
       </c>
-      <c r="H112" s="621"/>
+      <c r="H112" s="619"/>
       <c r="I112" s="502"/>
-      <c r="J112" s="621" t="s">
+      <c r="J112" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="K112" s="621"/>
-      <c r="L112" s="621"/>
-      <c r="M112" s="621"/>
-      <c r="N112" s="621"/>
-      <c r="O112" s="621"/>
-      <c r="P112" s="624" t="s">
+      <c r="K112" s="619"/>
+      <c r="L112" s="619"/>
+      <c r="M112" s="619"/>
+      <c r="N112" s="619"/>
+      <c r="O112" s="619"/>
+      <c r="P112" s="625" t="s">
         <v>218</v>
       </c>
       <c r="Q112" s="367"/>
     </row>
     <row r="113" spans="2:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B113" s="620"/>
-      <c r="C113" s="621"/>
-      <c r="D113" s="621"/>
-      <c r="E113" s="621"/>
-      <c r="F113" s="621"/>
+      <c r="B113" s="628"/>
+      <c r="C113" s="619"/>
+      <c r="D113" s="619"/>
+      <c r="E113" s="619"/>
+      <c r="F113" s="619"/>
       <c r="G113" s="583">
         <v>2027</v>
       </c>
@@ -14022,7 +14086,7 @@
       <c r="O113" s="445">
         <v>2030</v>
       </c>
-      <c r="P113" s="625"/>
+      <c r="P113" s="626"/>
       <c r="Q113" s="367"/>
     </row>
     <row r="114" spans="2:17" ht="30" x14ac:dyDescent="0.25">
@@ -14072,85 +14136,6 @@
     </row>
   </sheetData>
   <mergeCells count="95">
-    <mergeCell ref="L3:Q3"/>
-    <mergeCell ref="R3:R4"/>
-    <mergeCell ref="J15:O15"/>
-    <mergeCell ref="P15:P16"/>
-    <mergeCell ref="J60:O60"/>
-    <mergeCell ref="P60:P61"/>
-    <mergeCell ref="J25:O25"/>
-    <mergeCell ref="P25:P26"/>
-    <mergeCell ref="J35:O35"/>
-    <mergeCell ref="P35:P36"/>
-    <mergeCell ref="J73:O73"/>
-    <mergeCell ref="P73:P74"/>
-    <mergeCell ref="J81:O81"/>
-    <mergeCell ref="P81:P82"/>
-    <mergeCell ref="J46:O46"/>
-    <mergeCell ref="P46:P47"/>
-    <mergeCell ref="B106:D106"/>
-    <mergeCell ref="J112:O112"/>
-    <mergeCell ref="P112:P113"/>
-    <mergeCell ref="B80:C80"/>
-    <mergeCell ref="J94:O94"/>
-    <mergeCell ref="P94:P95"/>
-    <mergeCell ref="J107:O107"/>
-    <mergeCell ref="P107:P108"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G15:H15"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:H25"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G35:H35"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="F81:F82"/>
-    <mergeCell ref="G60:H60"/>
-    <mergeCell ref="B73:B74"/>
-    <mergeCell ref="C73:C74"/>
-    <mergeCell ref="D73:D74"/>
-    <mergeCell ref="E73:E74"/>
-    <mergeCell ref="F73:F74"/>
-    <mergeCell ref="G73:H73"/>
-    <mergeCell ref="B60:B61"/>
-    <mergeCell ref="C60:C61"/>
-    <mergeCell ref="D60:D61"/>
-    <mergeCell ref="E60:E61"/>
-    <mergeCell ref="F60:F61"/>
-    <mergeCell ref="G112:H112"/>
-    <mergeCell ref="B107:B108"/>
-    <mergeCell ref="C107:C108"/>
-    <mergeCell ref="D107:D108"/>
-    <mergeCell ref="E107:E108"/>
-    <mergeCell ref="F107:F108"/>
-    <mergeCell ref="B111:D111"/>
-    <mergeCell ref="B112:B113"/>
-    <mergeCell ref="C112:C113"/>
-    <mergeCell ref="D112:D113"/>
-    <mergeCell ref="E112:E113"/>
-    <mergeCell ref="F112:F113"/>
     <mergeCell ref="B1:H1"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="K3:K4"/>
@@ -14167,6 +14152,85 @@
     <mergeCell ref="C81:C82"/>
     <mergeCell ref="D81:D82"/>
     <mergeCell ref="E81:E82"/>
+    <mergeCell ref="B112:B113"/>
+    <mergeCell ref="C112:C113"/>
+    <mergeCell ref="D112:D113"/>
+    <mergeCell ref="E112:E113"/>
+    <mergeCell ref="F112:F113"/>
+    <mergeCell ref="G60:H60"/>
+    <mergeCell ref="B73:B74"/>
+    <mergeCell ref="C73:C74"/>
+    <mergeCell ref="D73:D74"/>
+    <mergeCell ref="E73:E74"/>
+    <mergeCell ref="F73:F74"/>
+    <mergeCell ref="G73:H73"/>
+    <mergeCell ref="B60:B61"/>
+    <mergeCell ref="C60:C61"/>
+    <mergeCell ref="D60:D61"/>
+    <mergeCell ref="E60:E61"/>
+    <mergeCell ref="F60:F61"/>
+    <mergeCell ref="G35:H35"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="G15:H15"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:H25"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="B106:D106"/>
+    <mergeCell ref="J112:O112"/>
+    <mergeCell ref="P112:P113"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="J94:O94"/>
+    <mergeCell ref="P94:P95"/>
+    <mergeCell ref="J107:O107"/>
+    <mergeCell ref="P107:P108"/>
+    <mergeCell ref="F81:F82"/>
+    <mergeCell ref="G112:H112"/>
+    <mergeCell ref="B107:B108"/>
+    <mergeCell ref="C107:C108"/>
+    <mergeCell ref="D107:D108"/>
+    <mergeCell ref="E107:E108"/>
+    <mergeCell ref="F107:F108"/>
+    <mergeCell ref="B111:D111"/>
+    <mergeCell ref="J73:O73"/>
+    <mergeCell ref="P73:P74"/>
+    <mergeCell ref="J81:O81"/>
+    <mergeCell ref="P81:P82"/>
+    <mergeCell ref="J46:O46"/>
+    <mergeCell ref="P46:P47"/>
+    <mergeCell ref="L3:Q3"/>
+    <mergeCell ref="R3:R4"/>
+    <mergeCell ref="J15:O15"/>
+    <mergeCell ref="P15:P16"/>
+    <mergeCell ref="J60:O60"/>
+    <mergeCell ref="P60:P61"/>
+    <mergeCell ref="J25:O25"/>
+    <mergeCell ref="P25:P26"/>
+    <mergeCell ref="J35:O35"/>
+    <mergeCell ref="P35:P36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -14194,46 +14258,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B1" s="638" t="s">
+      <c r="B1" s="648" t="s">
         <v>308</v>
       </c>
-      <c r="C1" s="638"/>
-      <c r="D1" s="638"/>
-      <c r="E1" s="638"/>
+      <c r="C1" s="648"/>
+      <c r="D1" s="648"/>
+      <c r="E1" s="648"/>
       <c r="F1" s="447"/>
       <c r="G1" s="447"/>
       <c r="J1" s="489"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B3" s="639" t="s">
+      <c r="B3" s="643" t="s">
         <v>309</v>
       </c>
-      <c r="C3" s="639"/>
-      <c r="D3" s="639"/>
-      <c r="E3" s="639"/>
-      <c r="F3" s="639"/>
-      <c r="G3" s="639"/>
-      <c r="H3" s="639"/>
+      <c r="C3" s="643"/>
+      <c r="D3" s="643"/>
+      <c r="E3" s="643"/>
+      <c r="F3" s="643"/>
+      <c r="G3" s="643"/>
+      <c r="H3" s="643"/>
       <c r="I3" s="581"/>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="447"/>
-      <c r="B4" s="637" t="s">
+      <c r="B4" s="642" t="s">
         <v>310</v>
       </c>
-      <c r="C4" s="637"/>
-      <c r="D4" s="637"/>
-      <c r="E4" s="637"/>
-      <c r="F4" s="637"/>
-      <c r="G4" s="637"/>
-      <c r="H4" s="637"/>
+      <c r="C4" s="642"/>
+      <c r="D4" s="642"/>
+      <c r="E4" s="642"/>
+      <c r="F4" s="642"/>
+      <c r="G4" s="642"/>
+      <c r="H4" s="642"/>
       <c r="I4" s="580"/>
     </row>
     <row r="5" spans="1:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="636" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="631" t="s">
+      <c r="C5" s="649" t="s">
         <v>311</v>
       </c>
       <c r="D5" s="636" t="s">
@@ -14253,21 +14317,21 @@
       </c>
       <c r="I5" s="636"/>
       <c r="J5" s="491"/>
-      <c r="K5" s="648" t="s">
+      <c r="K5" s="631" t="s">
         <v>217</v>
       </c>
-      <c r="L5" s="649"/>
-      <c r="M5" s="649"/>
-      <c r="N5" s="649"/>
-      <c r="O5" s="649"/>
-      <c r="P5" s="650"/>
-      <c r="Q5" s="640" t="s">
+      <c r="L5" s="632"/>
+      <c r="M5" s="632"/>
+      <c r="N5" s="632"/>
+      <c r="O5" s="632"/>
+      <c r="P5" s="633"/>
+      <c r="Q5" s="634" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="B6" s="636"/>
-      <c r="C6" s="632"/>
+      <c r="C6" s="650"/>
       <c r="D6" s="636"/>
       <c r="E6" s="636"/>
       <c r="F6" s="636"/>
@@ -14297,7 +14361,7 @@
       <c r="P6" s="448">
         <v>2030</v>
       </c>
-      <c r="Q6" s="641"/>
+      <c r="Q6" s="635"/>
     </row>
     <row r="7" spans="1:17" ht="22.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="543"/>
@@ -14338,7 +14402,7 @@
       <c r="B8" s="545">
         <v>1</v>
       </c>
-      <c r="C8" s="633" t="s">
+      <c r="C8" s="645" t="s">
         <v>312</v>
       </c>
       <c r="D8" s="544" t="s">
@@ -14377,7 +14441,7 @@
       <c r="B9" s="545">
         <v>2</v>
       </c>
-      <c r="C9" s="634"/>
+      <c r="C9" s="646"/>
       <c r="D9" s="546" t="s">
         <v>219</v>
       </c>
@@ -14422,7 +14486,7 @@
       <c r="B10" s="545">
         <v>4</v>
       </c>
-      <c r="C10" s="634"/>
+      <c r="C10" s="646"/>
       <c r="D10" s="544" t="s">
         <v>32</v>
       </c>
@@ -14459,7 +14523,7 @@
       <c r="B11" s="545">
         <v>5</v>
       </c>
-      <c r="C11" s="634"/>
+      <c r="C11" s="646"/>
       <c r="D11" s="546" t="s">
         <v>219</v>
       </c>
@@ -14504,7 +14568,7 @@
       <c r="B12" s="545">
         <v>6</v>
       </c>
-      <c r="C12" s="635"/>
+      <c r="C12" s="647"/>
       <c r="D12" s="546" t="s">
         <v>221</v>
       </c>
@@ -14546,22 +14610,22 @@
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="B14" s="637" t="s">
+      <c r="B14" s="642" t="s">
         <v>316</v>
       </c>
-      <c r="C14" s="637"/>
-      <c r="D14" s="637"/>
-      <c r="E14" s="637"/>
-      <c r="F14" s="637"/>
-      <c r="G14" s="637"/>
-      <c r="H14" s="637"/>
+      <c r="C14" s="642"/>
+      <c r="D14" s="642"/>
+      <c r="E14" s="642"/>
+      <c r="F14" s="642"/>
+      <c r="G14" s="642"/>
+      <c r="H14" s="642"/>
       <c r="I14" s="580"/>
     </row>
     <row r="15" spans="1:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="636" t="s">
         <v>48</v>
       </c>
-      <c r="C15" s="631" t="s">
+      <c r="C15" s="649" t="s">
         <v>311</v>
       </c>
       <c r="D15" s="636" t="s">
@@ -14581,21 +14645,21 @@
       </c>
       <c r="I15" s="636"/>
       <c r="J15" s="492"/>
-      <c r="K15" s="621" t="s">
+      <c r="K15" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L15" s="621"/>
-      <c r="M15" s="621"/>
-      <c r="N15" s="621"/>
-      <c r="O15" s="621"/>
-      <c r="P15" s="621"/>
-      <c r="Q15" s="642" t="s">
+      <c r="L15" s="619"/>
+      <c r="M15" s="619"/>
+      <c r="N15" s="619"/>
+      <c r="O15" s="619"/>
+      <c r="P15" s="619"/>
+      <c r="Q15" s="637" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="636"/>
-      <c r="C16" s="632"/>
+      <c r="C16" s="650"/>
       <c r="D16" s="636"/>
       <c r="E16" s="636"/>
       <c r="F16" s="636"/>
@@ -14625,7 +14689,7 @@
       <c r="P16" s="448">
         <v>2030</v>
       </c>
-      <c r="Q16" s="642"/>
+      <c r="Q16" s="637"/>
     </row>
     <row r="17" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B17" s="543"/>
@@ -14666,7 +14730,7 @@
       <c r="B18" s="547">
         <v>1</v>
       </c>
-      <c r="C18" s="633" t="s">
+      <c r="C18" s="645" t="s">
         <v>276</v>
       </c>
       <c r="D18" s="548" t="s">
@@ -14713,7 +14777,7 @@
       <c r="B19" s="547">
         <v>2</v>
       </c>
-      <c r="C19" s="634"/>
+      <c r="C19" s="646"/>
       <c r="D19" s="548" t="s">
         <v>30</v>
       </c>
@@ -14758,7 +14822,7 @@
       <c r="B20" s="547">
         <v>3</v>
       </c>
-      <c r="C20" s="634"/>
+      <c r="C20" s="646"/>
       <c r="D20" s="548" t="s">
         <v>317</v>
       </c>
@@ -14797,7 +14861,7 @@
       <c r="B21" s="547">
         <v>4</v>
       </c>
-      <c r="C21" s="634"/>
+      <c r="C21" s="646"/>
       <c r="D21" s="548" t="s">
         <v>31</v>
       </c>
@@ -14842,7 +14906,7 @@
       <c r="B22" s="547">
         <v>5</v>
       </c>
-      <c r="C22" s="635"/>
+      <c r="C22" s="647"/>
       <c r="D22" s="548" t="s">
         <v>318</v>
       </c>
@@ -14902,22 +14966,22 @@
       <c r="Q23" s="564"/>
     </row>
     <row r="24" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B24" s="637" t="s">
+      <c r="B24" s="642" t="s">
         <v>319</v>
       </c>
-      <c r="C24" s="637"/>
-      <c r="D24" s="637"/>
-      <c r="E24" s="637"/>
-      <c r="F24" s="637"/>
-      <c r="G24" s="637"/>
-      <c r="H24" s="637"/>
+      <c r="C24" s="642"/>
+      <c r="D24" s="642"/>
+      <c r="E24" s="642"/>
+      <c r="F24" s="642"/>
+      <c r="G24" s="642"/>
+      <c r="H24" s="642"/>
       <c r="I24" s="580"/>
     </row>
     <row r="25" spans="2:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="636" t="s">
         <v>48</v>
       </c>
-      <c r="C25" s="631" t="s">
+      <c r="C25" s="649" t="s">
         <v>311</v>
       </c>
       <c r="D25" s="636" t="s">
@@ -14937,21 +15001,21 @@
       </c>
       <c r="I25" s="636"/>
       <c r="J25" s="492"/>
-      <c r="K25" s="621" t="s">
+      <c r="K25" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L25" s="621"/>
-      <c r="M25" s="621"/>
-      <c r="N25" s="621"/>
-      <c r="O25" s="621"/>
-      <c r="P25" s="621"/>
-      <c r="Q25" s="640" t="s">
+      <c r="L25" s="619"/>
+      <c r="M25" s="619"/>
+      <c r="N25" s="619"/>
+      <c r="O25" s="619"/>
+      <c r="P25" s="619"/>
+      <c r="Q25" s="634" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="26" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B26" s="636"/>
-      <c r="C26" s="632"/>
+      <c r="C26" s="650"/>
       <c r="D26" s="636"/>
       <c r="E26" s="636"/>
       <c r="F26" s="636"/>
@@ -14981,7 +15045,7 @@
       <c r="P26" s="448">
         <v>2030</v>
       </c>
-      <c r="Q26" s="641"/>
+      <c r="Q26" s="635"/>
     </row>
     <row r="27" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B27" s="543"/>
@@ -15022,7 +15086,7 @@
       <c r="B28" s="547">
         <v>1</v>
       </c>
-      <c r="C28" s="633" t="s">
+      <c r="C28" s="645" t="s">
         <v>278</v>
       </c>
       <c r="D28" s="548" t="s">
@@ -15069,7 +15133,7 @@
       <c r="B29" s="547">
         <v>2</v>
       </c>
-      <c r="C29" s="634"/>
+      <c r="C29" s="646"/>
       <c r="D29" s="548" t="s">
         <v>28</v>
       </c>
@@ -15114,7 +15178,7 @@
       <c r="B30" s="547">
         <v>3</v>
       </c>
-      <c r="C30" s="634"/>
+      <c r="C30" s="646"/>
       <c r="D30" s="548" t="s">
         <v>30</v>
       </c>
@@ -15159,7 +15223,7 @@
       <c r="B31" s="547">
         <v>4</v>
       </c>
-      <c r="C31" s="634"/>
+      <c r="C31" s="646"/>
       <c r="D31" s="548" t="s">
         <v>317</v>
       </c>
@@ -15198,7 +15262,7 @@
       <c r="B32" s="547">
         <v>5</v>
       </c>
-      <c r="C32" s="634"/>
+      <c r="C32" s="646"/>
       <c r="D32" s="548" t="s">
         <v>31</v>
       </c>
@@ -15243,7 +15307,7 @@
       <c r="B33" s="547">
         <v>6</v>
       </c>
-      <c r="C33" s="635"/>
+      <c r="C33" s="647"/>
       <c r="D33" s="548" t="s">
         <v>318</v>
       </c>
@@ -15285,22 +15349,22 @@
       </c>
     </row>
     <row r="35" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B35" s="637" t="s">
+      <c r="B35" s="642" t="s">
         <v>321</v>
       </c>
-      <c r="C35" s="637"/>
-      <c r="D35" s="637"/>
-      <c r="E35" s="637"/>
-      <c r="F35" s="637"/>
-      <c r="G35" s="637"/>
-      <c r="H35" s="637"/>
+      <c r="C35" s="642"/>
+      <c r="D35" s="642"/>
+      <c r="E35" s="642"/>
+      <c r="F35" s="642"/>
+      <c r="G35" s="642"/>
+      <c r="H35" s="642"/>
       <c r="I35" s="580"/>
     </row>
     <row r="36" spans="2:18" ht="22.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="636" t="s">
         <v>48</v>
       </c>
-      <c r="C36" s="631" t="s">
+      <c r="C36" s="649" t="s">
         <v>311</v>
       </c>
       <c r="D36" s="636" t="s">
@@ -15320,21 +15384,21 @@
       </c>
       <c r="I36" s="636"/>
       <c r="J36" s="492"/>
-      <c r="K36" s="621" t="s">
+      <c r="K36" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L36" s="621"/>
-      <c r="M36" s="621"/>
-      <c r="N36" s="621"/>
-      <c r="O36" s="621"/>
-      <c r="P36" s="621"/>
-      <c r="Q36" s="640" t="s">
+      <c r="L36" s="619"/>
+      <c r="M36" s="619"/>
+      <c r="N36" s="619"/>
+      <c r="O36" s="619"/>
+      <c r="P36" s="619"/>
+      <c r="Q36" s="634" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="37" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B37" s="636"/>
-      <c r="C37" s="632"/>
+      <c r="C37" s="650"/>
       <c r="D37" s="636"/>
       <c r="E37" s="636"/>
       <c r="F37" s="636"/>
@@ -15364,7 +15428,7 @@
       <c r="P37" s="448">
         <v>2030</v>
       </c>
-      <c r="Q37" s="641"/>
+      <c r="Q37" s="635"/>
     </row>
     <row r="38" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B38" s="543"/>
@@ -15405,7 +15469,7 @@
       <c r="B39" s="547">
         <v>1</v>
       </c>
-      <c r="C39" s="633" t="s">
+      <c r="C39" s="645" t="s">
         <v>272</v>
       </c>
       <c r="D39" s="548" t="s">
@@ -15452,7 +15516,7 @@
       <c r="B40" s="547">
         <v>3</v>
       </c>
-      <c r="C40" s="634"/>
+      <c r="C40" s="646"/>
       <c r="D40" s="548" t="s">
         <v>30</v>
       </c>
@@ -15497,7 +15561,7 @@
       <c r="B41" s="547">
         <v>2</v>
       </c>
-      <c r="C41" s="634"/>
+      <c r="C41" s="646"/>
       <c r="D41" s="548" t="s">
         <v>317</v>
       </c>
@@ -15536,7 +15600,7 @@
       <c r="B42" s="547">
         <v>4</v>
       </c>
-      <c r="C42" s="634"/>
+      <c r="C42" s="646"/>
       <c r="D42" s="548" t="s">
         <v>31</v>
       </c>
@@ -15581,7 +15645,7 @@
       <c r="B43" s="547">
         <v>5</v>
       </c>
-      <c r="C43" s="635"/>
+      <c r="C43" s="647"/>
       <c r="D43" s="548" t="s">
         <v>318</v>
       </c>
@@ -15624,22 +15688,22 @@
       <c r="R43" s="471"/>
     </row>
     <row r="45" spans="2:18" x14ac:dyDescent="0.25">
-      <c r="B45" s="637" t="s">
+      <c r="B45" s="642" t="s">
         <v>322</v>
       </c>
-      <c r="C45" s="637"/>
-      <c r="D45" s="637"/>
-      <c r="E45" s="637"/>
-      <c r="F45" s="637"/>
-      <c r="G45" s="637"/>
-      <c r="H45" s="637"/>
+      <c r="C45" s="642"/>
+      <c r="D45" s="642"/>
+      <c r="E45" s="642"/>
+      <c r="F45" s="642"/>
+      <c r="G45" s="642"/>
+      <c r="H45" s="642"/>
       <c r="I45" s="580"/>
     </row>
     <row r="46" spans="2:18" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B46" s="636" t="s">
         <v>48</v>
       </c>
-      <c r="C46" s="631" t="s">
+      <c r="C46" s="649" t="s">
         <v>311</v>
       </c>
       <c r="D46" s="636" t="s">
@@ -15659,21 +15723,21 @@
       </c>
       <c r="I46" s="636"/>
       <c r="J46" s="492"/>
-      <c r="K46" s="621" t="s">
+      <c r="K46" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L46" s="621"/>
-      <c r="M46" s="621"/>
-      <c r="N46" s="621"/>
-      <c r="O46" s="621"/>
-      <c r="P46" s="621"/>
-      <c r="Q46" s="640" t="s">
+      <c r="L46" s="619"/>
+      <c r="M46" s="619"/>
+      <c r="N46" s="619"/>
+      <c r="O46" s="619"/>
+      <c r="P46" s="619"/>
+      <c r="Q46" s="634" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="47" spans="2:18" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="636"/>
-      <c r="C47" s="632"/>
+      <c r="C47" s="650"/>
       <c r="D47" s="636"/>
       <c r="E47" s="636"/>
       <c r="F47" s="636"/>
@@ -15703,7 +15767,7 @@
       <c r="P47" s="448">
         <v>2030</v>
       </c>
-      <c r="Q47" s="641"/>
+      <c r="Q47" s="635"/>
     </row>
     <row r="48" spans="2:18" x14ac:dyDescent="0.25">
       <c r="B48" s="449"/>
@@ -15744,7 +15808,7 @@
       <c r="B49" s="547">
         <v>1</v>
       </c>
-      <c r="C49" s="633" t="s">
+      <c r="C49" s="645" t="s">
         <v>274</v>
       </c>
       <c r="D49" s="548" t="s">
@@ -15783,7 +15847,7 @@
       <c r="B50" s="547">
         <v>2</v>
       </c>
-      <c r="C50" s="634"/>
+      <c r="C50" s="646"/>
       <c r="D50" s="548" t="s">
         <v>28</v>
       </c>
@@ -15822,7 +15886,7 @@
       <c r="B51" s="547">
         <v>3</v>
       </c>
-      <c r="C51" s="634"/>
+      <c r="C51" s="646"/>
       <c r="D51" s="548" t="s">
         <v>30</v>
       </c>
@@ -15861,7 +15925,7 @@
       <c r="B52" s="547">
         <v>4</v>
       </c>
-      <c r="C52" s="634"/>
+      <c r="C52" s="646"/>
       <c r="D52" s="548" t="s">
         <v>317</v>
       </c>
@@ -15900,7 +15964,7 @@
       <c r="B53" s="547">
         <v>5</v>
       </c>
-      <c r="C53" s="634"/>
+      <c r="C53" s="646"/>
       <c r="D53" s="548" t="s">
         <v>31</v>
       </c>
@@ -15937,7 +16001,7 @@
       <c r="B54" s="547">
         <v>6</v>
       </c>
-      <c r="C54" s="635"/>
+      <c r="C54" s="647"/>
       <c r="D54" s="548" t="s">
         <v>318</v>
       </c>
@@ -15971,34 +16035,34 @@
       <c r="Q54" s="563"/>
     </row>
     <row r="57" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B57" s="639" t="s">
+      <c r="B57" s="643" t="s">
         <v>323</v>
       </c>
-      <c r="C57" s="639"/>
-      <c r="D57" s="639"/>
-      <c r="E57" s="639"/>
-      <c r="F57" s="639"/>
-      <c r="G57" s="639"/>
-      <c r="H57" s="639"/>
+      <c r="C57" s="643"/>
+      <c r="D57" s="643"/>
+      <c r="E57" s="643"/>
+      <c r="F57" s="643"/>
+      <c r="G57" s="643"/>
+      <c r="H57" s="643"/>
       <c r="I57" s="581"/>
     </row>
     <row r="58" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B58" s="637" t="s">
+      <c r="B58" s="642" t="s">
         <v>324</v>
       </c>
-      <c r="C58" s="637"/>
-      <c r="D58" s="637"/>
-      <c r="E58" s="637"/>
-      <c r="F58" s="637"/>
-      <c r="G58" s="637"/>
-      <c r="H58" s="637"/>
+      <c r="C58" s="642"/>
+      <c r="D58" s="642"/>
+      <c r="E58" s="642"/>
+      <c r="F58" s="642"/>
+      <c r="G58" s="642"/>
+      <c r="H58" s="642"/>
       <c r="I58" s="580"/>
     </row>
     <row r="59" spans="2:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B59" s="636" t="s">
         <v>48</v>
       </c>
-      <c r="C59" s="631" t="s">
+      <c r="C59" s="649" t="s">
         <v>311</v>
       </c>
       <c r="D59" s="636" t="s">
@@ -16018,21 +16082,21 @@
       </c>
       <c r="I59" s="636"/>
       <c r="J59" s="492"/>
-      <c r="K59" s="621" t="s">
+      <c r="K59" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L59" s="621"/>
-      <c r="M59" s="621"/>
-      <c r="N59" s="621"/>
-      <c r="O59" s="621"/>
-      <c r="P59" s="621"/>
-      <c r="Q59" s="640" t="s">
+      <c r="L59" s="619"/>
+      <c r="M59" s="619"/>
+      <c r="N59" s="619"/>
+      <c r="O59" s="619"/>
+      <c r="P59" s="619"/>
+      <c r="Q59" s="634" t="s">
         <v>218</v>
       </c>
     </row>
     <row r="60" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B60" s="636"/>
-      <c r="C60" s="632"/>
+      <c r="C60" s="650"/>
       <c r="D60" s="636"/>
       <c r="E60" s="636"/>
       <c r="F60" s="636"/>
@@ -16062,7 +16126,7 @@
       <c r="P60" s="448">
         <v>2030</v>
       </c>
-      <c r="Q60" s="641"/>
+      <c r="Q60" s="635"/>
     </row>
     <row r="61" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B61" s="543"/>
@@ -16103,7 +16167,7 @@
       <c r="B62" s="547">
         <v>1</v>
       </c>
-      <c r="C62" s="633" t="s">
+      <c r="C62" s="645" t="s">
         <v>325</v>
       </c>
       <c r="D62" s="548" t="s">
@@ -16150,7 +16214,7 @@
       <c r="B63" s="547">
         <v>2</v>
       </c>
-      <c r="C63" s="634"/>
+      <c r="C63" s="646"/>
       <c r="D63" s="548" t="s">
         <v>328</v>
       </c>
@@ -16193,7 +16257,7 @@
     </row>
     <row r="64" spans="2:17" ht="34.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B64" s="547"/>
-      <c r="C64" s="634"/>
+      <c r="C64" s="646"/>
       <c r="D64" s="548" t="s">
         <v>330</v>
       </c>
@@ -16238,7 +16302,7 @@
       <c r="B65" s="547">
         <v>4</v>
       </c>
-      <c r="C65" s="634"/>
+      <c r="C65" s="646"/>
       <c r="D65" s="548" t="s">
         <v>30</v>
       </c>
@@ -16283,7 +16347,7 @@
       <c r="B66" s="547">
         <v>5</v>
       </c>
-      <c r="C66" s="634"/>
+      <c r="C66" s="646"/>
       <c r="D66" s="548" t="s">
         <v>317</v>
       </c>
@@ -16322,7 +16386,7 @@
       <c r="B67" s="547">
         <v>6</v>
       </c>
-      <c r="C67" s="635"/>
+      <c r="C67" s="647"/>
       <c r="D67" s="548" t="s">
         <v>31</v>
       </c>
@@ -16364,27 +16428,27 @@
       </c>
     </row>
     <row r="69" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B69" s="639" t="s">
+      <c r="B69" s="643" t="s">
         <v>331</v>
       </c>
-      <c r="C69" s="639"/>
-      <c r="D69" s="639"/>
-      <c r="E69" s="639"/>
-      <c r="F69" s="639"/>
-      <c r="G69" s="639"/>
-      <c r="H69" s="639"/>
+      <c r="C69" s="643"/>
+      <c r="D69" s="643"/>
+      <c r="E69" s="643"/>
+      <c r="F69" s="643"/>
+      <c r="G69" s="643"/>
+      <c r="H69" s="643"/>
       <c r="I69" s="581"/>
     </row>
     <row r="70" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B70" s="637" t="s">
+      <c r="B70" s="642" t="s">
         <v>332</v>
       </c>
-      <c r="C70" s="637"/>
-      <c r="D70" s="637"/>
-      <c r="E70" s="637"/>
-      <c r="F70" s="637"/>
-      <c r="G70" s="637"/>
-      <c r="H70" s="637"/>
+      <c r="C70" s="642"/>
+      <c r="D70" s="642"/>
+      <c r="E70" s="642"/>
+      <c r="F70" s="642"/>
+      <c r="G70" s="642"/>
+      <c r="H70" s="642"/>
       <c r="I70" s="580"/>
     </row>
     <row r="71" spans="2:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -16411,15 +16475,15 @@
       </c>
       <c r="I71" s="636"/>
       <c r="J71" s="492"/>
-      <c r="K71" s="621" t="s">
+      <c r="K71" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L71" s="621"/>
-      <c r="M71" s="621"/>
-      <c r="N71" s="621"/>
-      <c r="O71" s="621"/>
-      <c r="P71" s="621"/>
-      <c r="Q71" s="640" t="s">
+      <c r="L71" s="619"/>
+      <c r="M71" s="619"/>
+      <c r="N71" s="619"/>
+      <c r="O71" s="619"/>
+      <c r="P71" s="619"/>
+      <c r="Q71" s="634" t="s">
         <v>218</v>
       </c>
     </row>
@@ -16455,7 +16519,7 @@
       <c r="P72" s="448">
         <v>2030</v>
       </c>
-      <c r="Q72" s="641"/>
+      <c r="Q72" s="635"/>
     </row>
     <row r="73" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B73" s="543"/>
@@ -16585,15 +16649,15 @@
       </c>
     </row>
     <row r="77" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B77" s="639" t="s">
+      <c r="B77" s="643" t="s">
         <v>335</v>
       </c>
-      <c r="C77" s="639"/>
-      <c r="D77" s="639"/>
-      <c r="E77" s="639"/>
-      <c r="F77" s="639"/>
-      <c r="G77" s="639"/>
-      <c r="H77" s="639"/>
+      <c r="C77" s="643"/>
+      <c r="D77" s="643"/>
+      <c r="E77" s="643"/>
+      <c r="F77" s="643"/>
+      <c r="G77" s="643"/>
+      <c r="H77" s="643"/>
       <c r="I77" s="581"/>
     </row>
     <row r="78" spans="2:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -16606,15 +16670,15 @@
       <c r="H78" s="500"/>
       <c r="I78" s="500"/>
       <c r="J78" s="492"/>
-      <c r="K78" s="621" t="s">
+      <c r="K78" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L78" s="621"/>
-      <c r="M78" s="621"/>
-      <c r="N78" s="621"/>
-      <c r="O78" s="621"/>
-      <c r="P78" s="621"/>
-      <c r="Q78" s="640" t="s">
+      <c r="L78" s="619"/>
+      <c r="M78" s="619"/>
+      <c r="N78" s="619"/>
+      <c r="O78" s="619"/>
+      <c r="P78" s="619"/>
+      <c r="Q78" s="634" t="s">
         <v>218</v>
       </c>
     </row>
@@ -16662,7 +16726,7 @@
       <c r="P79" s="448">
         <v>2030</v>
       </c>
-      <c r="Q79" s="641"/>
+      <c r="Q79" s="635"/>
     </row>
     <row r="80" spans="2:17" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B80" s="543"/>
@@ -16703,7 +16767,7 @@
       <c r="B81" s="545">
         <v>1</v>
       </c>
-      <c r="C81" s="643" t="s">
+      <c r="C81" s="638" t="s">
         <v>336</v>
       </c>
       <c r="D81" s="552" t="s">
@@ -16744,7 +16808,7 @@
       <c r="B82" s="545">
         <v>2</v>
       </c>
-      <c r="C82" s="643"/>
+      <c r="C82" s="638"/>
       <c r="D82" s="552" t="s">
         <v>338</v>
       </c>
@@ -16783,7 +16847,7 @@
       <c r="B83" s="545">
         <v>3</v>
       </c>
-      <c r="C83" s="643"/>
+      <c r="C83" s="638"/>
       <c r="D83" s="552" t="s">
         <v>160</v>
       </c>
@@ -16855,27 +16919,27 @@
       <c r="Q85" s="565"/>
     </row>
     <row r="86" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B86" s="639" t="s">
+      <c r="B86" s="643" t="s">
         <v>339</v>
       </c>
-      <c r="C86" s="639"/>
-      <c r="D86" s="639"/>
-      <c r="E86" s="639"/>
-      <c r="F86" s="639"/>
-      <c r="G86" s="639"/>
-      <c r="H86" s="639"/>
+      <c r="C86" s="643"/>
+      <c r="D86" s="643"/>
+      <c r="E86" s="643"/>
+      <c r="F86" s="643"/>
+      <c r="G86" s="643"/>
+      <c r="H86" s="643"/>
       <c r="I86" s="581"/>
     </row>
     <row r="87" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B87" s="637" t="s">
+      <c r="B87" s="642" t="s">
         <v>287</v>
       </c>
-      <c r="C87" s="637"/>
-      <c r="D87" s="637"/>
-      <c r="E87" s="637"/>
-      <c r="F87" s="637"/>
-      <c r="G87" s="637"/>
-      <c r="H87" s="637"/>
+      <c r="C87" s="642"/>
+      <c r="D87" s="642"/>
+      <c r="E87" s="642"/>
+      <c r="F87" s="642"/>
+      <c r="G87" s="642"/>
+      <c r="H87" s="642"/>
       <c r="I87" s="580"/>
     </row>
     <row r="88" spans="2:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -16902,15 +16966,15 @@
       </c>
       <c r="I88" s="636"/>
       <c r="J88" s="492"/>
-      <c r="K88" s="621" t="s">
+      <c r="K88" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L88" s="621"/>
-      <c r="M88" s="621"/>
-      <c r="N88" s="621"/>
-      <c r="O88" s="621"/>
-      <c r="P88" s="621"/>
-      <c r="Q88" s="640" t="s">
+      <c r="L88" s="619"/>
+      <c r="M88" s="619"/>
+      <c r="N88" s="619"/>
+      <c r="O88" s="619"/>
+      <c r="P88" s="619"/>
+      <c r="Q88" s="634" t="s">
         <v>218</v>
       </c>
     </row>
@@ -16946,7 +17010,7 @@
       <c r="P89" s="448">
         <v>2030</v>
       </c>
-      <c r="Q89" s="641"/>
+      <c r="Q89" s="635"/>
     </row>
     <row r="90" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B90" s="543"/>
@@ -16987,7 +17051,7 @@
       <c r="B91" s="545">
         <v>1</v>
       </c>
-      <c r="C91" s="643" t="s">
+      <c r="C91" s="638" t="s">
         <v>287</v>
       </c>
       <c r="D91" s="552" t="s">
@@ -17034,7 +17098,7 @@
       <c r="B92" s="545">
         <v>2</v>
       </c>
-      <c r="C92" s="643"/>
+      <c r="C92" s="638"/>
       <c r="D92" s="552" t="s">
         <v>28</v>
       </c>
@@ -17079,7 +17143,7 @@
       <c r="B93" s="545">
         <v>3</v>
       </c>
-      <c r="C93" s="643"/>
+      <c r="C93" s="638"/>
       <c r="D93" s="552" t="s">
         <v>341</v>
       </c>
@@ -17122,7 +17186,7 @@
     </row>
     <row r="94" spans="2:17" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B94" s="545"/>
-      <c r="C94" s="643"/>
+      <c r="C94" s="638"/>
       <c r="D94" s="552" t="s">
         <v>342</v>
       </c>
@@ -17159,7 +17223,7 @@
       <c r="B95" s="545">
         <v>4</v>
       </c>
-      <c r="C95" s="643"/>
+      <c r="C95" s="638"/>
       <c r="D95" s="552" t="s">
         <v>21</v>
       </c>
@@ -17202,7 +17266,7 @@
     </row>
     <row r="96" spans="2:17" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B96" s="545"/>
-      <c r="C96" s="643"/>
+      <c r="C96" s="638"/>
       <c r="D96" s="552" t="s">
         <v>31</v>
       </c>
@@ -17247,7 +17311,7 @@
       <c r="B97" s="545">
         <v>5</v>
       </c>
-      <c r="C97" s="643"/>
+      <c r="C97" s="638"/>
       <c r="D97" s="552" t="s">
         <v>318</v>
       </c>
@@ -17287,15 +17351,15 @@
       <c r="Q97" s="563"/>
     </row>
     <row r="99" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B99" s="637" t="s">
+      <c r="B99" s="642" t="s">
         <v>344</v>
       </c>
-      <c r="C99" s="637"/>
-      <c r="D99" s="637"/>
-      <c r="E99" s="637"/>
-      <c r="F99" s="637"/>
-      <c r="G99" s="637"/>
-      <c r="H99" s="637"/>
+      <c r="C99" s="642"/>
+      <c r="D99" s="642"/>
+      <c r="E99" s="642"/>
+      <c r="F99" s="642"/>
+      <c r="G99" s="642"/>
+      <c r="H99" s="642"/>
       <c r="I99" s="580"/>
     </row>
     <row r="100" spans="2:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -17322,15 +17386,15 @@
       </c>
       <c r="I100" s="636"/>
       <c r="J100" s="492"/>
-      <c r="K100" s="621" t="s">
+      <c r="K100" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L100" s="621"/>
-      <c r="M100" s="621"/>
-      <c r="N100" s="621"/>
-      <c r="O100" s="621"/>
-      <c r="P100" s="621"/>
-      <c r="Q100" s="640" t="s">
+      <c r="L100" s="619"/>
+      <c r="M100" s="619"/>
+      <c r="N100" s="619"/>
+      <c r="O100" s="619"/>
+      <c r="P100" s="619"/>
+      <c r="Q100" s="634" t="s">
         <v>218</v>
       </c>
     </row>
@@ -17366,7 +17430,7 @@
       <c r="P101" s="448">
         <v>2030</v>
       </c>
-      <c r="Q101" s="641"/>
+      <c r="Q101" s="635"/>
     </row>
     <row r="102" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B102" s="543"/>
@@ -17407,7 +17471,7 @@
       <c r="B103" s="545">
         <v>1</v>
       </c>
-      <c r="C103" s="645" t="s">
+      <c r="C103" s="639" t="s">
         <v>233</v>
       </c>
       <c r="D103" s="555" t="s">
@@ -17454,7 +17518,7 @@
       <c r="B104" s="545">
         <v>2</v>
       </c>
-      <c r="C104" s="646"/>
+      <c r="C104" s="640"/>
       <c r="D104" s="555" t="s">
         <v>28</v>
       </c>
@@ -17499,7 +17563,7 @@
       <c r="B105" s="545">
         <v>3</v>
       </c>
-      <c r="C105" s="646"/>
+      <c r="C105" s="640"/>
       <c r="D105" s="555" t="s">
         <v>341</v>
       </c>
@@ -17544,7 +17608,7 @@
       <c r="B106" s="545">
         <v>4</v>
       </c>
-      <c r="C106" s="646"/>
+      <c r="C106" s="640"/>
       <c r="D106" s="555" t="s">
         <v>342</v>
       </c>
@@ -17575,7 +17639,7 @@
       <c r="B107" s="545">
         <v>5</v>
       </c>
-      <c r="C107" s="646"/>
+      <c r="C107" s="640"/>
       <c r="D107" s="555" t="s">
         <v>31</v>
       </c>
@@ -17620,7 +17684,7 @@
       <c r="B108" s="545">
         <v>6</v>
       </c>
-      <c r="C108" s="646"/>
+      <c r="C108" s="640"/>
       <c r="D108" s="555" t="s">
         <v>21</v>
       </c>
@@ -17665,7 +17729,7 @@
       <c r="B109" s="545">
         <v>7</v>
       </c>
-      <c r="C109" s="647"/>
+      <c r="C109" s="641"/>
       <c r="D109" s="555" t="s">
         <v>318</v>
       </c>
@@ -17707,15 +17771,15 @@
       </c>
     </row>
     <row r="111" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B111" s="637" t="s">
+      <c r="B111" s="642" t="s">
         <v>348</v>
       </c>
-      <c r="C111" s="637"/>
-      <c r="D111" s="637"/>
-      <c r="E111" s="637"/>
-      <c r="F111" s="637"/>
-      <c r="G111" s="637"/>
-      <c r="H111" s="637"/>
+      <c r="C111" s="642"/>
+      <c r="D111" s="642"/>
+      <c r="E111" s="642"/>
+      <c r="F111" s="642"/>
+      <c r="G111" s="642"/>
+      <c r="H111" s="642"/>
       <c r="I111" s="580"/>
     </row>
     <row r="112" spans="2:17" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -17742,15 +17806,15 @@
       </c>
       <c r="I112" s="636"/>
       <c r="J112" s="492"/>
-      <c r="K112" s="621" t="s">
+      <c r="K112" s="619" t="s">
         <v>217</v>
       </c>
-      <c r="L112" s="621"/>
-      <c r="M112" s="621"/>
-      <c r="N112" s="621"/>
-      <c r="O112" s="621"/>
-      <c r="P112" s="621"/>
-      <c r="Q112" s="642" t="s">
+      <c r="L112" s="619"/>
+      <c r="M112" s="619"/>
+      <c r="N112" s="619"/>
+      <c r="O112" s="619"/>
+      <c r="P112" s="619"/>
+      <c r="Q112" s="637" t="s">
         <v>218</v>
       </c>
     </row>
@@ -17786,7 +17850,7 @@
       <c r="P113" s="448">
         <v>2030</v>
       </c>
-      <c r="Q113" s="642"/>
+      <c r="Q113" s="637"/>
     </row>
     <row r="114" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B114" s="543"/>
@@ -17827,7 +17891,7 @@
       <c r="B115" s="545">
         <v>1</v>
       </c>
-      <c r="C115" s="643" t="s">
+      <c r="C115" s="638" t="s">
         <v>160</v>
       </c>
       <c r="D115" s="555" t="s">
@@ -17874,7 +17938,7 @@
       <c r="B116" s="545">
         <v>2</v>
       </c>
-      <c r="C116" s="643"/>
+      <c r="C116" s="638"/>
       <c r="D116" s="555" t="s">
         <v>28</v>
       </c>
@@ -17917,7 +17981,7 @@
       <c r="B117" s="545">
         <v>3</v>
       </c>
-      <c r="C117" s="643"/>
+      <c r="C117" s="638"/>
       <c r="D117" s="555" t="s">
         <v>341</v>
       </c>
@@ -17962,7 +18026,7 @@
       <c r="B118" s="545">
         <v>4</v>
       </c>
-      <c r="C118" s="643"/>
+      <c r="C118" s="638"/>
       <c r="D118" s="555" t="s">
         <v>342</v>
       </c>
@@ -18001,7 +18065,7 @@
       <c r="B119" s="545">
         <v>5</v>
       </c>
-      <c r="C119" s="643"/>
+      <c r="C119" s="638"/>
       <c r="D119" s="555" t="s">
         <v>31</v>
       </c>
@@ -18044,7 +18108,7 @@
       <c r="B120" s="545">
         <v>6</v>
       </c>
-      <c r="C120" s="643"/>
+      <c r="C120" s="638"/>
       <c r="D120" s="555" t="s">
         <v>21</v>
       </c>
@@ -18089,7 +18153,7 @@
       <c r="B121" s="545">
         <v>7</v>
       </c>
-      <c r="C121" s="643"/>
+      <c r="C121" s="638"/>
       <c r="D121" s="555" t="s">
         <v>325</v>
       </c>
@@ -18142,18 +18206,89 @@
     </row>
   </sheetData>
   <mergeCells count="119">
-    <mergeCell ref="K15:P15"/>
-    <mergeCell ref="K5:P5"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="Q15:Q16"/>
-    <mergeCell ref="F15:F16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="B112:B113"/>
+    <mergeCell ref="C112:C113"/>
+    <mergeCell ref="D112:D113"/>
+    <mergeCell ref="B46:B47"/>
+    <mergeCell ref="C46:C47"/>
+    <mergeCell ref="D46:D47"/>
+    <mergeCell ref="B87:H87"/>
+    <mergeCell ref="B88:B89"/>
+    <mergeCell ref="C88:C89"/>
+    <mergeCell ref="D88:D89"/>
+    <mergeCell ref="E88:E89"/>
+    <mergeCell ref="F88:F89"/>
+    <mergeCell ref="B99:H99"/>
+    <mergeCell ref="B111:H111"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="C49:C54"/>
+    <mergeCell ref="C39:C43"/>
+    <mergeCell ref="C28:C33"/>
+    <mergeCell ref="C18:C22"/>
+    <mergeCell ref="C8:C12"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G59:G60"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="B71:B72"/>
+    <mergeCell ref="C71:C72"/>
+    <mergeCell ref="D71:D72"/>
+    <mergeCell ref="E71:E72"/>
+    <mergeCell ref="F71:F72"/>
+    <mergeCell ref="G71:G72"/>
+    <mergeCell ref="H71:I71"/>
+    <mergeCell ref="B59:B60"/>
+    <mergeCell ref="C59:C60"/>
+    <mergeCell ref="D59:D60"/>
+    <mergeCell ref="E59:E60"/>
+    <mergeCell ref="F59:F60"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B14:H14"/>
+    <mergeCell ref="B4:H4"/>
+    <mergeCell ref="B3:H3"/>
+    <mergeCell ref="B57:H57"/>
+    <mergeCell ref="B58:H58"/>
+    <mergeCell ref="B35:H35"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="E46:E47"/>
+    <mergeCell ref="F46:F47"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:C37"/>
+    <mergeCell ref="D36:D37"/>
+    <mergeCell ref="E36:E37"/>
+    <mergeCell ref="F36:F37"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="Q88:Q89"/>
+    <mergeCell ref="Q100:Q101"/>
+    <mergeCell ref="Q112:Q113"/>
+    <mergeCell ref="B45:H45"/>
+    <mergeCell ref="B70:H70"/>
+    <mergeCell ref="B69:H69"/>
+    <mergeCell ref="B77:H77"/>
+    <mergeCell ref="Q71:Q72"/>
+    <mergeCell ref="K112:P112"/>
+    <mergeCell ref="K78:P78"/>
+    <mergeCell ref="C81:C83"/>
+    <mergeCell ref="K71:P71"/>
+    <mergeCell ref="C74:C75"/>
+    <mergeCell ref="K59:P59"/>
+    <mergeCell ref="C62:C67"/>
+    <mergeCell ref="B86:H86"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="E112:E113"/>
+    <mergeCell ref="F112:F113"/>
+    <mergeCell ref="B100:B101"/>
+    <mergeCell ref="C100:C101"/>
+    <mergeCell ref="D100:D101"/>
+    <mergeCell ref="E100:E101"/>
+    <mergeCell ref="F100:F101"/>
     <mergeCell ref="Q25:Q26"/>
     <mergeCell ref="Q36:Q37"/>
     <mergeCell ref="Q46:Q47"/>
@@ -18178,89 +18313,18 @@
     <mergeCell ref="G36:G37"/>
     <mergeCell ref="H36:I36"/>
     <mergeCell ref="G46:G47"/>
-    <mergeCell ref="Q88:Q89"/>
-    <mergeCell ref="Q100:Q101"/>
-    <mergeCell ref="Q112:Q113"/>
-    <mergeCell ref="B45:H45"/>
-    <mergeCell ref="B70:H70"/>
-    <mergeCell ref="B69:H69"/>
-    <mergeCell ref="B77:H77"/>
-    <mergeCell ref="Q71:Q72"/>
-    <mergeCell ref="K112:P112"/>
-    <mergeCell ref="K78:P78"/>
-    <mergeCell ref="C81:C83"/>
-    <mergeCell ref="K71:P71"/>
-    <mergeCell ref="C74:C75"/>
-    <mergeCell ref="K59:P59"/>
-    <mergeCell ref="C62:C67"/>
-    <mergeCell ref="B86:H86"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B14:H14"/>
-    <mergeCell ref="B4:H4"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B57:H57"/>
-    <mergeCell ref="B58:H58"/>
-    <mergeCell ref="B35:H35"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="E46:E47"/>
-    <mergeCell ref="F46:F47"/>
-    <mergeCell ref="B36:B37"/>
-    <mergeCell ref="C36:C37"/>
-    <mergeCell ref="D36:D37"/>
-    <mergeCell ref="E36:E37"/>
-    <mergeCell ref="F36:F37"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G59:G60"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="B71:B72"/>
-    <mergeCell ref="C71:C72"/>
-    <mergeCell ref="D71:D72"/>
-    <mergeCell ref="E71:E72"/>
-    <mergeCell ref="F71:F72"/>
-    <mergeCell ref="G71:G72"/>
-    <mergeCell ref="H71:I71"/>
-    <mergeCell ref="B59:B60"/>
-    <mergeCell ref="C59:C60"/>
-    <mergeCell ref="D59:D60"/>
-    <mergeCell ref="E59:E60"/>
-    <mergeCell ref="F59:F60"/>
-    <mergeCell ref="E112:E113"/>
-    <mergeCell ref="F112:F113"/>
-    <mergeCell ref="B100:B101"/>
-    <mergeCell ref="C100:C101"/>
-    <mergeCell ref="D100:D101"/>
-    <mergeCell ref="E100:E101"/>
-    <mergeCell ref="F100:F101"/>
-    <mergeCell ref="B88:B89"/>
-    <mergeCell ref="C88:C89"/>
-    <mergeCell ref="D88:D89"/>
-    <mergeCell ref="E88:E89"/>
-    <mergeCell ref="F88:F89"/>
-    <mergeCell ref="B99:H99"/>
-    <mergeCell ref="B111:H111"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="C49:C54"/>
-    <mergeCell ref="C39:C43"/>
-    <mergeCell ref="C28:C33"/>
-    <mergeCell ref="C18:C22"/>
-    <mergeCell ref="C8:C12"/>
-    <mergeCell ref="B112:B113"/>
-    <mergeCell ref="C112:C113"/>
-    <mergeCell ref="D112:D113"/>
-    <mergeCell ref="B46:B47"/>
-    <mergeCell ref="C46:C47"/>
-    <mergeCell ref="D46:D47"/>
-    <mergeCell ref="B87:H87"/>
+    <mergeCell ref="K15:P15"/>
+    <mergeCell ref="K5:P5"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="Q15:Q16"/>
+    <mergeCell ref="F15:F16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:I15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
@@ -18268,6 +18332,501 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="6" width="9" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="14.140625" customWidth="1"/>
+    <col min="10" max="10" width="13.140625" customWidth="1"/>
+    <col min="11" max="11" width="19.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A1" s="663"/>
+      <c r="B1" s="663" t="s">
+        <v>352</v>
+      </c>
+      <c r="C1" s="664" t="s">
+        <v>355</v>
+      </c>
+      <c r="D1" s="664"/>
+      <c r="E1" s="664"/>
+      <c r="F1" s="664" t="s">
+        <v>353</v>
+      </c>
+      <c r="G1" s="664"/>
+      <c r="H1" s="664"/>
+      <c r="I1" s="665" t="s">
+        <v>356</v>
+      </c>
+      <c r="J1" s="667"/>
+      <c r="K1" s="666"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="663" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="663"/>
+      <c r="C2" s="663" t="s">
+        <v>354</v>
+      </c>
+      <c r="D2" s="663">
+        <v>2027</v>
+      </c>
+      <c r="E2" s="663">
+        <v>2028</v>
+      </c>
+      <c r="F2" s="663" t="s">
+        <v>354</v>
+      </c>
+      <c r="G2" s="663">
+        <v>2027</v>
+      </c>
+      <c r="H2" s="663">
+        <v>2028</v>
+      </c>
+      <c r="I2" s="663" t="s">
+        <v>354</v>
+      </c>
+      <c r="J2" s="663">
+        <v>2027</v>
+      </c>
+      <c r="K2" s="663">
+        <v>2028</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="668"/>
+      <c r="B3" s="668" t="s">
+        <v>360</v>
+      </c>
+      <c r="C3" s="669">
+        <f>SUBTOTAL(9,C4:C15)</f>
+        <v>0</v>
+      </c>
+      <c r="D3" s="669">
+        <f>SUBTOTAL(9,D4:D15)</f>
+        <v>0</v>
+      </c>
+      <c r="E3" s="669">
+        <f>SUBTOTAL(9,E4:E15)</f>
+        <v>0</v>
+      </c>
+      <c r="F3" s="669">
+        <f>SUBTOTAL(9,F4:F15)</f>
+        <v>0</v>
+      </c>
+      <c r="G3" s="669">
+        <f>SUBTOTAL(9,G4:G15)</f>
+        <v>0</v>
+      </c>
+      <c r="H3" s="669">
+        <f>SUBTOTAL(9,H4:H15)</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="669"/>
+      <c r="J3" s="669"/>
+      <c r="K3" s="669"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="375">
+        <v>1</v>
+      </c>
+      <c r="B4" s="662" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="670">
+        <f>SUM(D4:E4)</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="670">
+        <f>'TH theo DV'!D4</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="670">
+        <f>'TH theo DV'!N4</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="670"/>
+      <c r="G4" s="670"/>
+      <c r="H4" s="670"/>
+      <c r="I4" s="662">
+        <f>C4-F4</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="662">
+        <f>D4-G4</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="662">
+        <f>E4-H4</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="375">
+        <v>2</v>
+      </c>
+      <c r="B5" s="662" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="670">
+        <f t="shared" ref="C5:C15" si="0">SUM(D5:E5)</f>
+        <v>0</v>
+      </c>
+      <c r="D5" s="670">
+        <f>'TH theo DV'!E4</f>
+        <v>0</v>
+      </c>
+      <c r="E5" s="670">
+        <f>'TH theo DV'!O4</f>
+        <v>0</v>
+      </c>
+      <c r="F5" s="670"/>
+      <c r="G5" s="670"/>
+      <c r="H5" s="670"/>
+      <c r="I5" s="662">
+        <f t="shared" ref="I5:I15" si="1">C5-F5</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="662">
+        <f t="shared" ref="J5:J15" si="2">D5-G5</f>
+        <v>0</v>
+      </c>
+      <c r="K5" s="662">
+        <f t="shared" ref="K5:K15" si="3">E5-H5</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="375">
+        <v>3</v>
+      </c>
+      <c r="B6" s="662" t="s">
+        <v>362</v>
+      </c>
+      <c r="C6" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D6" s="670">
+        <f>'TH theo DV'!F4</f>
+        <v>0</v>
+      </c>
+      <c r="E6" s="670">
+        <f>'TH theo DV'!P4</f>
+        <v>0</v>
+      </c>
+      <c r="F6" s="670"/>
+      <c r="G6" s="670"/>
+      <c r="H6" s="670"/>
+      <c r="I6" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J6" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K6" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="375">
+        <v>4</v>
+      </c>
+      <c r="B7" s="662" t="s">
+        <v>357</v>
+      </c>
+      <c r="C7" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D7" s="671"/>
+      <c r="E7" s="671"/>
+      <c r="F7" s="670"/>
+      <c r="G7" s="670"/>
+      <c r="H7" s="670"/>
+      <c r="I7" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J7" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K7" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="375">
+        <v>5</v>
+      </c>
+      <c r="B8" s="662" t="s">
+        <v>120</v>
+      </c>
+      <c r="C8" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D8" s="671"/>
+      <c r="E8" s="671"/>
+      <c r="F8" s="670"/>
+      <c r="G8" s="670"/>
+      <c r="H8" s="670"/>
+      <c r="I8" s="662">
+        <f>C8-F8</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="662">
+        <f>D8-G8</f>
+        <v>0</v>
+      </c>
+      <c r="K8" s="662">
+        <f>E8-H8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A9" s="375">
+        <v>6</v>
+      </c>
+      <c r="B9" s="662" t="s">
+        <v>361</v>
+      </c>
+      <c r="C9" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D9" s="671"/>
+      <c r="E9" s="671"/>
+      <c r="F9" s="670"/>
+      <c r="G9" s="670"/>
+      <c r="H9" s="670"/>
+      <c r="I9" s="662">
+        <f>C9-F9</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="662">
+        <f>D9-G9</f>
+        <v>0</v>
+      </c>
+      <c r="K9" s="662">
+        <f>E9-H9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A10" s="375">
+        <v>7</v>
+      </c>
+      <c r="B10" s="662" t="s">
+        <v>208</v>
+      </c>
+      <c r="C10" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D10" s="671"/>
+      <c r="E10" s="671"/>
+      <c r="F10" s="670"/>
+      <c r="G10" s="670"/>
+      <c r="H10" s="670"/>
+      <c r="I10" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J10" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K10" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A11" s="375">
+        <v>8</v>
+      </c>
+      <c r="B11" s="662" t="s">
+        <v>341</v>
+      </c>
+      <c r="C11" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D11" s="670">
+        <f>'TH theo DV'!H4</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="670">
+        <f>'TH theo DV'!R4</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="670"/>
+      <c r="G11" s="670"/>
+      <c r="H11" s="670"/>
+      <c r="I11" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J11" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K11" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A12" s="375">
+        <v>9</v>
+      </c>
+      <c r="B12" s="662" t="s">
+        <v>342</v>
+      </c>
+      <c r="C12" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D12" s="670">
+        <f>'TH theo DV'!I4</f>
+        <v>0</v>
+      </c>
+      <c r="E12" s="670">
+        <f>'TH theo DV'!S4</f>
+        <v>0</v>
+      </c>
+      <c r="F12" s="670"/>
+      <c r="G12" s="670"/>
+      <c r="H12" s="670"/>
+      <c r="I12" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J12" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K12" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A13" s="375">
+        <v>10</v>
+      </c>
+      <c r="B13" s="662" t="s">
+        <v>358</v>
+      </c>
+      <c r="C13" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D13" s="671"/>
+      <c r="E13" s="671"/>
+      <c r="F13" s="670"/>
+      <c r="G13" s="670"/>
+      <c r="H13" s="670"/>
+      <c r="I13" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J13" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K13" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A14" s="375">
+        <v>11</v>
+      </c>
+      <c r="B14" s="662" t="s">
+        <v>359</v>
+      </c>
+      <c r="C14" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D14" s="671"/>
+      <c r="E14" s="671"/>
+      <c r="F14" s="670"/>
+      <c r="G14" s="670"/>
+      <c r="H14" s="670"/>
+      <c r="I14" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J14" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K14" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A15" s="375">
+        <v>12</v>
+      </c>
+      <c r="B15" s="662" t="s">
+        <v>318</v>
+      </c>
+      <c r="C15" s="670">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="D15" s="670">
+        <f>'TH theo DV'!K4</f>
+        <v>0</v>
+      </c>
+      <c r="E15" s="670">
+        <f>'TH theo DV'!U4</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="670"/>
+      <c r="G15" s="670"/>
+      <c r="H15" s="670"/>
+      <c r="I15" s="662">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="J15" s="662">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="K15" s="662">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="I1:K1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet4">
     <tabColor rgb="FFEE0033"/>
@@ -20441,7 +21000,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet2">
     <tabColor rgb="FFEE0033"/>
@@ -21084,7 +21643,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet6"/>
   <dimension ref="B2:K35"/>

</xml_diff>